<commit_message>
refactor: aclarar columnas de excels
</commit_message>
<xml_diff>
--- a/input/zips.xlsx
+++ b/input/zips.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="zips" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="zips" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,18 +413,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>nombre</t>
+          <t>pagina_origen</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>url</t>
+          <t>nombre_zip</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>url_zip</t>
         </is>
       </c>
     </row>

</xml_diff>